<commit_message>
fix(ui): polish mobile design, add footer, Hindi guidance hints, and fix ACCOUNT typo in excel template
</commit_message>
<xml_diff>
--- a/templates/DPO_Muzaffarpur_Arrear_Forms.xlsx
+++ b/templates/DPO_Muzaffarpur_Arrear_Forms.xlsx
@@ -736,7 +736,7 @@
       <c r="H5" s="17" t="n"/>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>ACCOUN NO.-</t>
+          <t>ACCOUNT NO.-</t>
         </is>
       </c>
       <c r="J5" s="16" t="n"/>
@@ -1520,7 +1520,7 @@
       <c r="E5" s="17" t="n"/>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>ACCOUN NO.-</t>
+          <t>ACCOUNT NO.-</t>
         </is>
       </c>
       <c r="G5" s="16" t="n"/>

</xml_diff>